<commit_message>
chore: sync data sources spreadsheet
</commit_message>
<xml_diff>
--- a/Partner School Success Dashboard Data Sources.xlsx
+++ b/Partner School Success Dashboard Data Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\Documents\PAMF\Pessoal\Professional\AI_Native_Journey\Mizuho Bank SMB Docs\Patner School Success Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D40BE1-FC3A-4D84-9554-E12C2A442357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39EF766-AA64-4662-B116-9FDD9DE3400D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data Sources" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <sheet name="Worked Examples" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2096,18 +2095,10 @@
     <xf numFmtId="10" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2116,6 +2107,14 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7576,26 +7575,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>446</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="54" t="s">
         <v>447</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
@@ -7610,12 +7609,12 @@
       <c r="A4" s="65" t="s">
         <v>448</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
@@ -8497,12 +8496,12 @@
       <c r="A49" s="66" t="s">
         <v>482</v>
       </c>
-      <c r="B49" s="54"/>
-      <c r="C49" s="54"/>
-      <c r="D49" s="54"/>
-      <c r="E49" s="54"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="54"/>
+      <c r="B49" s="51"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
@@ -8517,12 +8516,12 @@
       <c r="A51" s="65" t="s">
         <v>483</v>
       </c>
-      <c r="B51" s="54"/>
-      <c r="C51" s="54"/>
-      <c r="D51" s="54"/>
-      <c r="E51" s="54"/>
-      <c r="F51" s="54"/>
-      <c r="G51" s="54"/>
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
+      <c r="E51" s="51"/>
+      <c r="F51" s="51"/>
+      <c r="G51" s="51"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
@@ -9404,12 +9403,12 @@
       <c r="A96" s="66" t="s">
         <v>494</v>
       </c>
-      <c r="B96" s="54"/>
-      <c r="C96" s="54"/>
-      <c r="D96" s="54"/>
-      <c r="E96" s="54"/>
-      <c r="F96" s="54"/>
-      <c r="G96" s="54"/>
+      <c r="B96" s="51"/>
+      <c r="C96" s="51"/>
+      <c r="D96" s="51"/>
+      <c r="E96" s="51"/>
+      <c r="F96" s="51"/>
+      <c r="G96" s="51"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="5"/>
@@ -9424,12 +9423,12 @@
       <c r="A98" s="66" t="s">
         <v>495</v>
       </c>
-      <c r="B98" s="54"/>
-      <c r="C98" s="54"/>
-      <c r="D98" s="54"/>
-      <c r="E98" s="54"/>
-      <c r="F98" s="54"/>
-      <c r="G98" s="54"/>
+      <c r="B98" s="51"/>
+      <c r="C98" s="51"/>
+      <c r="D98" s="51"/>
+      <c r="E98" s="51"/>
+      <c r="F98" s="51"/>
+      <c r="G98" s="51"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="5"/>
@@ -9444,12 +9443,12 @@
       <c r="A100" s="65" t="s">
         <v>496</v>
       </c>
-      <c r="B100" s="54"/>
-      <c r="C100" s="54"/>
-      <c r="D100" s="54"/>
-      <c r="E100" s="54"/>
-      <c r="F100" s="54"/>
-      <c r="G100" s="54"/>
+      <c r="B100" s="51"/>
+      <c r="C100" s="51"/>
+      <c r="D100" s="51"/>
+      <c r="E100" s="51"/>
+      <c r="F100" s="51"/>
+      <c r="G100" s="51"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="5"/>
@@ -10331,12 +10330,12 @@
       <c r="A145" s="66" t="s">
         <v>500</v>
       </c>
-      <c r="B145" s="54"/>
-      <c r="C145" s="54"/>
-      <c r="D145" s="54"/>
-      <c r="E145" s="54"/>
-      <c r="F145" s="54"/>
-      <c r="G145" s="54"/>
+      <c r="B145" s="51"/>
+      <c r="C145" s="51"/>
+      <c r="D145" s="51"/>
+      <c r="E145" s="51"/>
+      <c r="F145" s="51"/>
+      <c r="G145" s="51"/>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="5"/>
@@ -10351,12 +10350,12 @@
       <c r="A147" s="66" t="s">
         <v>501</v>
       </c>
-      <c r="B147" s="54"/>
-      <c r="C147" s="54"/>
-      <c r="D147" s="54"/>
-      <c r="E147" s="54"/>
-      <c r="F147" s="54"/>
-      <c r="G147" s="54"/>
+      <c r="B147" s="51"/>
+      <c r="C147" s="51"/>
+      <c r="D147" s="51"/>
+      <c r="E147" s="51"/>
+      <c r="F147" s="51"/>
+      <c r="G147" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -10416,22 +10415,22 @@
       <c r="H1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="53" t="s">
+      <c r="J1" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="54"/>
+      <c r="K1" s="51"/>
     </row>
     <row r="2" spans="1:25" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="52"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="57"/>
       <c r="J2" s="14" t="s">
         <v>8</v>
       </c>
@@ -10501,16 +10500,16 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="52"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="57"/>
       <c r="J6" s="14" t="s">
         <v>11</v>
       </c>
@@ -11044,16 +11043,16 @@
       <c r="K29" s="6"/>
     </row>
     <row r="30" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="51"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="51"/>
-      <c r="G30" s="51"/>
-      <c r="H30" s="52"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="57"/>
       <c r="K30" s="6"/>
     </row>
     <row r="31" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11388,16 +11387,16 @@
       <c r="K46" s="6"/>
     </row>
     <row r="47" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="50" t="s">
+      <c r="A47" s="55" t="s">
         <v>218</v>
       </c>
-      <c r="B47" s="51"/>
-      <c r="C47" s="51"/>
-      <c r="D47" s="51"/>
-      <c r="E47" s="51"/>
-      <c r="F47" s="51"/>
-      <c r="G47" s="51"/>
-      <c r="H47" s="52"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="56"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="57"/>
       <c r="K47" s="6"/>
     </row>
     <row r="48" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11724,16 +11723,16 @@
       <c r="K61" s="6"/>
     </row>
     <row r="62" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="50" t="s">
+      <c r="A62" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="B62" s="51"/>
-      <c r="C62" s="51"/>
-      <c r="D62" s="51"/>
-      <c r="E62" s="51"/>
-      <c r="F62" s="51"/>
-      <c r="G62" s="51"/>
-      <c r="H62" s="52"/>
+      <c r="B62" s="56"/>
+      <c r="C62" s="56"/>
+      <c r="D62" s="56"/>
+      <c r="E62" s="56"/>
+      <c r="F62" s="56"/>
+      <c r="G62" s="56"/>
+      <c r="H62" s="57"/>
       <c r="K62" s="6"/>
     </row>
     <row r="63" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11979,16 +11978,16 @@
       <c r="K73" s="6"/>
     </row>
     <row r="74" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="50" t="s">
+      <c r="A74" s="55" t="s">
         <v>341</v>
       </c>
-      <c r="B74" s="51"/>
-      <c r="C74" s="51"/>
-      <c r="D74" s="51"/>
-      <c r="E74" s="51"/>
-      <c r="F74" s="51"/>
-      <c r="G74" s="51"/>
-      <c r="H74" s="52"/>
+      <c r="B74" s="56"/>
+      <c r="C74" s="56"/>
+      <c r="D74" s="56"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="57"/>
       <c r="K74" s="6"/>
     </row>
     <row r="75" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -12191,16 +12190,16 @@
       <c r="K86" s="6"/>
     </row>
     <row r="87" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="50" t="s">
+      <c r="A87" s="55" t="s">
         <v>353</v>
       </c>
-      <c r="B87" s="51"/>
-      <c r="C87" s="51"/>
-      <c r="D87" s="51"/>
-      <c r="E87" s="51"/>
-      <c r="F87" s="51"/>
-      <c r="G87" s="51"/>
-      <c r="H87" s="52"/>
+      <c r="B87" s="56"/>
+      <c r="C87" s="56"/>
+      <c r="D87" s="56"/>
+      <c r="E87" s="56"/>
+      <c r="F87" s="56"/>
+      <c r="G87" s="56"/>
+      <c r="H87" s="57"/>
       <c r="K87" s="6"/>
     </row>
     <row r="88" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -17702,12 +17701,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
@@ -17732,16 +17731,16 @@
       <c r="Z1" s="6"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
@@ -17848,16 +17847,16 @@
       <c r="Z5" s="6"/>
     </row>
     <row r="6" spans="1:26" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
       <c r="I6" s="19"/>
       <c r="J6" s="19"/>
       <c r="K6" s="19"/>
@@ -17878,16 +17877,16 @@
       <c r="Z6" s="19"/>
     </row>
     <row r="7" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
+      <c r="B7" s="51"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="51"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="51"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
       <c r="K7" s="19"/>
@@ -17908,16 +17907,16 @@
       <c r="Z7" s="19"/>
     </row>
     <row r="8" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
       <c r="K8" s="19"/>
@@ -17938,16 +17937,16 @@
       <c r="Z8" s="19"/>
     </row>
     <row r="9" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="55" t="s">
+      <c r="A9" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
@@ -17968,16 +17967,16 @@
       <c r="Z9" s="19"/>
     </row>
     <row r="10" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="55" t="s">
+      <c r="A10" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
       <c r="I10" s="19"/>
       <c r="J10" s="19"/>
       <c r="K10" s="19"/>
@@ -17998,16 +17997,16 @@
       <c r="Z10" s="19"/>
     </row>
     <row r="11" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="55" t="s">
+      <c r="A11" s="50" t="s">
         <v>97</v>
       </c>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
+      <c r="B11" s="51"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="51"/>
+      <c r="E11" s="51"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="51"/>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
       <c r="K11" s="19"/>
@@ -18346,16 +18345,16 @@
       <c r="Z21" s="6"/>
     </row>
     <row r="22" spans="1:26" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="56" t="s">
+      <c r="A22" s="52" t="s">
         <v>190</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+      <c r="H22" s="51"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -18376,16 +18375,16 @@
       <c r="Z22" s="13"/>
     </row>
     <row r="23" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="56" t="s">
+      <c r="A23" s="52" t="s">
         <v>192</v>
       </c>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54"/>
-      <c r="H23" s="54"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
       <c r="I23" s="13"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
@@ -18465,14 +18464,14 @@
       <c r="A3" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -18627,14 +18626,14 @@
       <c r="A8" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
@@ -18912,14 +18911,14 @@
       <c r="A15" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
@@ -19080,14 +19079,14 @@
       <c r="A19" s="60" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="54"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
-      <c r="H19" s="54"/>
-      <c r="I19" s="54"/>
+      <c r="B19" s="51"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
@@ -19138,14 +19137,14 @@
       <c r="A21" s="61" t="s">
         <v>155</v>
       </c>
-      <c r="B21" s="54"/>
-      <c r="C21" s="54"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="51"/>
+      <c r="I21" s="51"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
@@ -19352,14 +19351,14 @@
       <c r="A26" s="60" t="s">
         <v>188</v>
       </c>
-      <c r="B26" s="54"/>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
-      <c r="I26" s="54"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
       <c r="L26" s="6"/>
@@ -19405,30 +19404,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="54" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
@@ -19445,14 +19444,14 @@
       <c r="A4" s="61" t="s">
         <v>221</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="51"/>
+      <c r="I4" s="51"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
@@ -19673,14 +19672,14 @@
       <c r="A13" s="61" t="s">
         <v>264</v>
       </c>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
@@ -19818,14 +19817,14 @@
       <c r="A18" s="61" t="s">
         <v>284</v>
       </c>
-      <c r="B18" s="54"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
+      <c r="B18" s="51"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="51"/>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
@@ -19952,14 +19951,14 @@
       <c r="A22" s="60" t="s">
         <v>309</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="54"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+      <c r="H22" s="51"/>
+      <c r="I22" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -19988,23 +19987,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="62" t="s">
         <v>285</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="51"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -20260,17 +20259,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>380</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="62" t="s">
         <v>381</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="51"/>
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -20282,8 +20281,8 @@
       <c r="A4" s="63" t="s">
         <v>382</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
@@ -20543,8 +20542,8 @@
       <c r="A14" s="63" t="s">
         <v>397</v>
       </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
@@ -20702,8 +20701,8 @@
       <c r="A21" s="63" t="s">
         <v>406</v>
       </c>
-      <c r="B21" s="54"/>
-      <c r="C21" s="54"/>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
@@ -20793,8 +20792,8 @@
       <c r="A26" s="63" t="s">
         <v>412</v>
       </c>
-      <c r="B26" s="54"/>
-      <c r="C26" s="54"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
@@ -20969,16 +20968,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>418</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="51"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="54" t="s">
         <v>419</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="51"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
@@ -21213,10 +21212,10 @@
       <c r="Z11" s="30"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="56" t="s">
+      <c r="A12" s="52" t="s">
         <v>434</v>
       </c>
-      <c r="B12" s="54"/>
+      <c r="B12" s="51"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
@@ -21274,7 +21273,7 @@
       <c r="A14" s="64" t="s">
         <v>435</v>
       </c>
-      <c r="B14" s="54"/>
+      <c r="B14" s="51"/>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
       <c r="E14" s="30"/>
@@ -21323,16 +21322,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="53" t="s">
         <v>436</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="51"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="62" t="s">
         <v>437</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="51"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>

</xml_diff>